<commit_message>
feat: aplicar reporte Jair 24-25/08 - gates Administrador, 409 en modales, alertas RAP_COMPARTIDO, accesos directos horarios, grilla por defecto
</commit_message>
<xml_diff>
--- a/backend/scripts/Plantilla_Importacion_CONINS.xlsx
+++ b/backend/scripts/Plantilla_Importacion_CONINS.xlsx
@@ -3,9 +3,10 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Grupos" sheetId="1" r:id="rId1"/>
-    <sheet name="Asignaciones" sheetId="2" r:id="rId2"/>
-    <sheet name="Horarios" sheetId="3" r:id="rId3"/>
+    <sheet name="Instructores" sheetId="1" r:id="rId1"/>
+    <sheet name="Grupos" sheetId="2" r:id="rId2"/>
+    <sheet name="Asignaciones" sheetId="3" r:id="rId3"/>
+    <sheet name="Horarios" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -399,6 +400,45 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>nombre</v>
+      </c>
+      <c r="B1" t="str">
+        <v>email</v>
+      </c>
+      <c r="C1" t="str">
+        <v>tipo_area</v>
+      </c>
+      <c r="D1" t="str">
+        <v>codigos_competencia</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Ana Perez</v>
+      </c>
+      <c r="B2" t="str">
+        <v>aperez@sena.edu.co</v>
+      </c>
+      <c r="C2" t="str">
+        <v>tecnica</v>
+      </c>
+      <c r="D2" t="str">
+        <v>38392,38376</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J2"/>
   <sheetData>
     <row r="1">
@@ -472,7 +512,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetData>
@@ -517,7 +557,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K2"/>
   <sheetData>

</xml_diff>